<commit_message>
Before the 614 meeting
</commit_message>
<xml_diff>
--- a/per_class.xlsx
+++ b/per_class.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/green/Downloads/multi_outputGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2B4A284-FB45-5A44-8ECB-648D120F66A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E123694-A982-3D4D-96B6-7D9191B67D73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="15980" xr2:uid="{B0103469-8E94-FF46-B664-11BDEEF6E197}"/>
+    <workbookView xWindow="740" yWindow="2300" windowWidth="28040" windowHeight="15980" xr2:uid="{B0103469-8E94-FF46-B664-11BDEEF6E197}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -296,11 +296,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -933,7 +934,7 @@
       <c r="R3">
         <v>101.86566892961601</v>
       </c>
-      <c r="S3">
+      <c r="S3" s="1">
         <v>419.78621635302397</v>
       </c>
       <c r="T3">
@@ -1001,7 +1002,7 @@
       <c r="B4">
         <v>9</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="1">
         <v>1</v>
       </c>
       <c r="D4">
@@ -1278,10 +1279,10 @@
       <c r="Q6">
         <v>914.46411132812398</v>
       </c>
-      <c r="R6">
+      <c r="R6" s="1">
         <v>1005.0124822998</v>
       </c>
-      <c r="S6">
+      <c r="S6" s="1">
         <v>2521.2215708894</v>
       </c>
       <c r="T6">
@@ -1293,13 +1294,13 @@
       <c r="V6">
         <v>0.98152935330082902</v>
       </c>
-      <c r="W6">
+      <c r="W6" s="1">
         <v>10.429636366417</v>
       </c>
       <c r="X6">
         <v>2.2606678007541898</v>
       </c>
-      <c r="Y6">
+      <c r="Y6" s="4">
         <v>1550.27544477688</v>
       </c>
       <c r="Z6">
@@ -1578,7 +1579,7 @@
       <c r="A9" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="2">
         <v>182</v>
       </c>
       <c r="C9">

</xml_diff>